<commit_message>
Add grading UI backed by color-tagged xlsx cells
Reads student names from column B and criteria from pale-blue label
cells on the evaluation sheet; joins metadata from criteres_reviewed.
Slider (0..1 step 0.25) writes into light-gray mark cells only.
Working copy lives in app-private storage; saves on nav and pause.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/26se_ba2_fire_evaluations_v1.16.xlsx
+++ b/26se_ba2_fire_evaluations_v1.16.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="W:\______FASTWORK______\EPFL\===E_FIRE2526===\evals\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{86902D24-03EC-4EBB-A4B5-4AD2855C6549}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{617E6B59-7E78-4360-9E45-D1D56F935DB6}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="43320" windowHeight="24640" xr2:uid="{9CF21808-12BF-6746-A432-FEE50409D437}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="10660" windowHeight="4900" xr2:uid="{9CF21808-12BF-6746-A432-FEE50409D437}"/>
   </bookViews>
   <sheets>
     <sheet name="evaluation" sheetId="1" r:id="rId1"/>
@@ -30,7 +30,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1055" uniqueCount="567">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1051" uniqueCount="566">
   <si>
     <t>NOM PRENOM</t>
   </si>
@@ -1371,9 +1371,6 @@
   </si>
   <si>
     <t>COEFF</t>
-  </si>
-  <si>
-    <t>cas par cas</t>
   </si>
   <si>
     <t>Paul</t>
@@ -21684,7 +21681,7 @@
       <c r="CJ1" s="126"/>
       <c r="CK1" s="104"/>
       <c r="CL1" s="109" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="CM1" s="124" t="s">
         <v>160</v>
@@ -21693,7 +21690,7 @@
         <v>216</v>
       </c>
       <c r="CO1" s="117" t="s">
-        <v>487</v>
+        <v>486</v>
       </c>
       <c r="CP1" s="118"/>
       <c r="CQ1" s="119"/>
@@ -21701,7 +21698,7 @@
     <row r="2" spans="1:95" ht="15" customHeight="1">
       <c r="A2" s="8"/>
       <c r="B2" s="113" t="s">
-        <v>488</v>
+        <v>487</v>
       </c>
       <c r="C2" s="127"/>
       <c r="D2" s="115">
@@ -21843,7 +21840,7 @@
     <row r="3" spans="1:95" ht="15" customHeight="1">
       <c r="A3" s="8"/>
       <c r="B3" s="113" t="s">
-        <v>566</v>
+        <v>565</v>
       </c>
       <c r="C3" s="114"/>
       <c r="D3" s="101" t="str">
@@ -21863,7 +21860,7 @@
         <v>G4</v>
       </c>
       <c r="H3" s="135" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="I3" s="101">
         <f>criteres_reviewed!$D$6</f>
@@ -21878,7 +21875,7 @@
         <v>3</v>
       </c>
       <c r="L3" s="135" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="M3" s="102">
         <f>criteres_reviewed!$D$9</f>
@@ -21901,7 +21898,7 @@
         <v>8</v>
       </c>
       <c r="R3" s="135" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="S3" s="102">
         <f>criteres_reviewed!$D$14</f>
@@ -21916,7 +21913,7 @@
         <v>11</v>
       </c>
       <c r="V3" s="135" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="W3" s="102">
         <f>criteres_reviewed!$D$17</f>
@@ -21935,7 +21932,7 @@
         <v>15</v>
       </c>
       <c r="AA3" s="135" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="AB3" s="102">
         <f>criteres_reviewed!$D$21</f>
@@ -21950,7 +21947,7 @@
         <v>18</v>
       </c>
       <c r="AE3" s="135" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="AF3" s="102">
         <f>criteres_reviewed!$D$24</f>
@@ -21965,7 +21962,7 @@
         <v>21</v>
       </c>
       <c r="AI3" s="135" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="AJ3" s="102">
         <f>criteres_reviewed!$D$27</f>
@@ -21976,7 +21973,7 @@
         <v>23</v>
       </c>
       <c r="AL3" s="135" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="AM3" s="102">
         <f>criteres_reviewed!$D$29</f>
@@ -21991,7 +21988,7 @@
         <v>26</v>
       </c>
       <c r="AP3" s="135" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="AQ3" s="102">
         <f>criteres_reviewed!$D$32</f>
@@ -22006,14 +22003,14 @@
         <v>29</v>
       </c>
       <c r="AT3" s="135" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="AU3" s="102">
         <f>criteres_reviewed!$D$35</f>
         <v>30</v>
       </c>
       <c r="AV3" s="135" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="AW3" s="102">
         <f>criteres_reviewed!$D$36</f>
@@ -22032,7 +22029,7 @@
         <v>34</v>
       </c>
       <c r="BA3" s="135" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="BB3" s="102">
         <f>criteres_reviewed!$D$40</f>
@@ -22055,7 +22052,7 @@
         <v>39</v>
       </c>
       <c r="BG3" s="135" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="BH3" s="102">
         <f>criteres_reviewed!$D$45</f>
@@ -22074,7 +22071,7 @@
         <v>43</v>
       </c>
       <c r="BL3" s="135" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="BM3" s="102">
         <f>criteres_reviewed!$D$49</f>
@@ -22097,7 +22094,7 @@
         <v>48</v>
       </c>
       <c r="BR3" s="135" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="BS3" s="102">
         <f>criteres_reviewed!$D$54</f>
@@ -22120,7 +22117,7 @@
         <v>53</v>
       </c>
       <c r="BX3" s="135" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="BY3" s="102">
         <f>criteres_reviewed!$D$59</f>
@@ -22131,7 +22128,7 @@
         <v>55</v>
       </c>
       <c r="CA3" s="135" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="CB3" s="102">
         <f>criteres_reviewed!$D$61</f>
@@ -22142,7 +22139,7 @@
         <v>57</v>
       </c>
       <c r="CD3" s="135" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="CE3" s="102">
         <f>criteres_reviewed!$D$63</f>
@@ -22153,7 +22150,7 @@
         <v>59</v>
       </c>
       <c r="CG3" s="135" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="CH3" s="102">
         <f>criteres_reviewed!$D$65</f>
@@ -22164,7 +22161,7 @@
         <v>61</v>
       </c>
       <c r="CJ3" s="135" t="s">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="CK3" s="105"/>
       <c r="CL3" s="110"/>
@@ -22181,15 +22178,19 @@
       </c>
       <c r="C4" s="114"/>
       <c r="D4" s="74">
+        <f>criteres_reviewed!$C$2</f>
         <v>1</v>
       </c>
       <c r="E4" s="76">
+        <f>criteres_reviewed!$C$3</f>
         <v>1</v>
       </c>
       <c r="F4" s="76">
+        <f>criteres_reviewed!$C$4</f>
         <v>1</v>
       </c>
       <c r="G4" s="76">
+        <f>criteres_reviewed!$C$5</f>
         <v>1</v>
       </c>
       <c r="H4" s="21">
@@ -23394,7 +23395,7 @@
         <v>0</v>
       </c>
       <c r="CM9" s="87" t="s">
-        <v>489</v>
+        <v>488</v>
       </c>
       <c r="CN9" s="81" t="s">
         <v>364</v>
@@ -23569,7 +23570,7 @@
         <v>0</v>
       </c>
       <c r="CM10" s="87" t="s">
-        <v>556</v>
+        <v>555</v>
       </c>
       <c r="CN10" s="82" t="s">
         <v>222</v>
@@ -24277,7 +24278,7 @@
         <v>0</v>
       </c>
       <c r="CM14" s="87" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
       <c r="CN14" s="82" t="s">
         <v>226</v>
@@ -24810,7 +24811,7 @@
         <v>0</v>
       </c>
       <c r="CM17" s="87" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="CN17" s="82" t="s">
         <v>229</v>
@@ -25164,7 +25165,7 @@
         <v>0</v>
       </c>
       <c r="CM19" s="87" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="CN19" s="84" t="s">
         <v>371</v>
@@ -25510,7 +25511,7 @@
         <v>0</v>
       </c>
       <c r="CM21" s="87" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="CN21" s="82" t="s">
         <v>231</v>
@@ -26558,7 +26559,7 @@
         <v>0</v>
       </c>
       <c r="CM27" s="87" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="CN27" s="82" t="s">
         <v>237</v>
@@ -26737,7 +26738,7 @@
         <v>0</v>
       </c>
       <c r="CM28" s="89" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="CN28" s="82" t="s">
         <v>238</v>
@@ -26916,7 +26917,7 @@
         <v>0</v>
       </c>
       <c r="CM29" s="89" t="s">
-        <v>495</v>
+        <v>494</v>
       </c>
       <c r="CN29" s="82" t="s">
         <v>239</v>
@@ -27095,7 +27096,7 @@
         <v>0</v>
       </c>
       <c r="CM30" s="89" t="s">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="CN30" s="82" t="s">
         <v>240</v>
@@ -27272,7 +27273,7 @@
         <v>0</v>
       </c>
       <c r="CM31" s="89" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="CN31" s="82" t="s">
         <v>241</v>
@@ -27449,7 +27450,7 @@
         <v>0</v>
       </c>
       <c r="CM32" s="89" t="s">
-        <v>498</v>
+        <v>497</v>
       </c>
       <c r="CN32" s="84" t="s">
         <v>370</v>
@@ -27624,7 +27625,7 @@
         <v>0</v>
       </c>
       <c r="CM33" s="89" t="s">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="CN33" s="82" t="s">
         <v>242</v>
@@ -27797,7 +27798,7 @@
         <v>0</v>
       </c>
       <c r="CM34" s="89" t="s">
-        <v>557</v>
+        <v>556</v>
       </c>
       <c r="CN34" s="82" t="s">
         <v>243</v>
@@ -27976,7 +27977,7 @@
         <v>0</v>
       </c>
       <c r="CM35" s="89" t="s">
-        <v>558</v>
+        <v>557</v>
       </c>
       <c r="CN35" s="82" t="s">
         <v>244</v>
@@ -28153,7 +28154,7 @@
         <v>0</v>
       </c>
       <c r="CM36" s="89" t="s">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="CN36" s="82" t="s">
         <v>245</v>
@@ -28328,7 +28329,7 @@
         <v>0</v>
       </c>
       <c r="CM37" s="89" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="CN37" s="82" t="s">
         <v>246</v>
@@ -28501,7 +28502,7 @@
         <v>0</v>
       </c>
       <c r="CM38" s="89" t="s">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="CN38" s="82" t="s">
         <v>247</v>
@@ -28855,7 +28856,7 @@
         <v>0</v>
       </c>
       <c r="CM40" s="89" t="s">
-        <v>503</v>
+        <v>502</v>
       </c>
       <c r="CN40" s="82" t="s">
         <v>249</v>
@@ -29030,7 +29031,7 @@
         <v>0</v>
       </c>
       <c r="CM41" s="89" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="CN41" s="82" t="s">
         <v>250</v>
@@ -29382,7 +29383,7 @@
         <v>0</v>
       </c>
       <c r="CM43" s="89" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="CN43" s="82" t="s">
         <v>252</v>
@@ -29557,7 +29558,7 @@
         <v>0</v>
       </c>
       <c r="CM44" s="89" t="s">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="CN44" s="82" t="s">
         <v>253</v>
@@ -29911,7 +29912,7 @@
         <v>0</v>
       </c>
       <c r="CM46" s="89" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="CN46" s="82" t="s">
         <v>255</v>
@@ -30090,7 +30091,7 @@
         <v>0</v>
       </c>
       <c r="CM47" s="89" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
       <c r="CN47" s="82" t="s">
         <v>256</v>
@@ -30269,7 +30270,7 @@
         <v>0</v>
       </c>
       <c r="CM48" s="89" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="CN48" s="82" t="s">
         <v>257</v>
@@ -30444,7 +30445,7 @@
         <v>0</v>
       </c>
       <c r="CM49" s="89" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="CN49" s="82" t="s">
         <v>282</v>
@@ -30621,7 +30622,7 @@
         <v>0</v>
       </c>
       <c r="CM50" s="89" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="CN50" s="82" t="s">
         <v>258</v>
@@ -30796,7 +30797,7 @@
         <v>0</v>
       </c>
       <c r="CM51" s="89" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="CN51" s="82" t="s">
         <v>323</v>
@@ -30975,7 +30976,7 @@
         <v>0</v>
       </c>
       <c r="CM52" s="89" t="s">
-        <v>559</v>
+        <v>558</v>
       </c>
       <c r="CN52" s="82" t="s">
         <v>324</v>
@@ -31148,7 +31149,7 @@
         <v>0</v>
       </c>
       <c r="CM53" s="89" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="CN53" s="82" t="s">
         <v>325</v>
@@ -31325,7 +31326,7 @@
         <v>0</v>
       </c>
       <c r="CM54" s="89" t="s">
-        <v>560</v>
+        <v>559</v>
       </c>
       <c r="CN54" s="82" t="s">
         <v>326</v>
@@ -31500,7 +31501,7 @@
         <v>0</v>
       </c>
       <c r="CM55" s="89" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="CN55" s="82" t="s">
         <v>327</v>
@@ -31679,7 +31680,7 @@
         <v>0</v>
       </c>
       <c r="CM56" s="89" t="s">
-        <v>514</v>
+        <v>513</v>
       </c>
       <c r="CN56" s="82" t="s">
         <v>259</v>
@@ -31854,7 +31855,7 @@
         <v>0</v>
       </c>
       <c r="CM57" s="89" t="s">
-        <v>515</v>
+        <v>514</v>
       </c>
       <c r="CN57" s="82" t="s">
         <v>328</v>
@@ -32033,7 +32034,7 @@
         <v>0</v>
       </c>
       <c r="CM58" s="89" t="s">
-        <v>516</v>
+        <v>515</v>
       </c>
       <c r="CN58" s="82" t="s">
         <v>329</v>
@@ -32212,7 +32213,7 @@
         <v>0</v>
       </c>
       <c r="CM59" s="89" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="CN59" s="82" t="s">
         <v>330</v>
@@ -32385,7 +32386,7 @@
         <v>0</v>
       </c>
       <c r="CM60" s="89" t="s">
-        <v>561</v>
+        <v>560</v>
       </c>
       <c r="CN60" s="82" t="s">
         <v>331</v>
@@ -32737,7 +32738,7 @@
         <v>0</v>
       </c>
       <c r="CM62" s="89" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="CN62" s="82" t="s">
         <v>333</v>
@@ -32916,7 +32917,7 @@
         <v>0</v>
       </c>
       <c r="CM63" s="89" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
       <c r="CN63" s="82" t="s">
         <v>334</v>
@@ -33095,7 +33096,7 @@
         <v>0</v>
       </c>
       <c r="CM64" s="89" t="s">
-        <v>562</v>
+        <v>561</v>
       </c>
       <c r="CN64" s="82" t="s">
         <v>335</v>
@@ -33441,7 +33442,7 @@
         <v>0</v>
       </c>
       <c r="CM66" s="89" t="s">
-        <v>520</v>
+        <v>519</v>
       </c>
       <c r="CN66" s="82" t="s">
         <v>337</v>
@@ -33618,7 +33619,7 @@
         <v>0</v>
       </c>
       <c r="CM67" s="89" t="s">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="CN67" s="82" t="s">
         <v>338</v>
@@ -33793,7 +33794,7 @@
         <v>0</v>
       </c>
       <c r="CM68" s="89" t="s">
-        <v>522</v>
+        <v>521</v>
       </c>
       <c r="CN68" s="82" t="s">
         <v>339</v>
@@ -33970,7 +33971,7 @@
         <v>0</v>
       </c>
       <c r="CM69" s="89" t="s">
-        <v>523</v>
+        <v>522</v>
       </c>
       <c r="CN69" s="82" t="s">
         <v>340</v>
@@ -34147,7 +34148,7 @@
         <v>0</v>
       </c>
       <c r="CM70" s="89" t="s">
-        <v>524</v>
+        <v>523</v>
       </c>
       <c r="CN70" s="82" t="s">
         <v>341</v>
@@ -34497,7 +34498,7 @@
         <v>0</v>
       </c>
       <c r="CM72" s="89" t="s">
-        <v>525</v>
+        <v>524</v>
       </c>
       <c r="CN72" s="82" t="s">
         <v>343</v>
@@ -34670,7 +34671,7 @@
         <v>0</v>
       </c>
       <c r="CM73" s="89" t="s">
-        <v>526</v>
+        <v>525</v>
       </c>
       <c r="CN73" s="82" t="s">
         <v>344</v>
@@ -35201,7 +35202,7 @@
         <v>0</v>
       </c>
       <c r="CM76" s="89" t="s">
-        <v>527</v>
+        <v>526</v>
       </c>
       <c r="CN76" s="82" t="s">
         <v>346</v>
@@ -35553,7 +35554,7 @@
         <v>0</v>
       </c>
       <c r="CM78" s="89" t="s">
-        <v>528</v>
+        <v>527</v>
       </c>
       <c r="CN78" s="82" t="s">
         <v>347</v>
@@ -37319,7 +37320,7 @@
         <v>0</v>
       </c>
       <c r="CM88" s="89" t="s">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="CN88" s="82" t="s">
         <v>355</v>
@@ -37494,7 +37495,7 @@
         <v>0</v>
       </c>
       <c r="CM89" s="89" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="CN89" s="82" t="s">
         <v>356</v>
@@ -38383,7 +38384,7 @@
         <v>0</v>
       </c>
       <c r="CM94" s="89" t="s">
-        <v>529</v>
+        <v>528</v>
       </c>
       <c r="CN94" s="82" t="s">
         <v>361</v>
@@ -38560,7 +38561,7 @@
         <v>0</v>
       </c>
       <c r="CM95" s="89" t="s">
-        <v>530</v>
+        <v>529</v>
       </c>
       <c r="CN95" s="82" t="s">
         <v>362</v>
@@ -39264,7 +39265,7 @@
         <v>0</v>
       </c>
       <c r="CM99" s="89" t="s">
-        <v>531</v>
+        <v>530</v>
       </c>
       <c r="CN99" s="82" t="s">
         <v>262</v>
@@ -39439,7 +39440,7 @@
         <v>0</v>
       </c>
       <c r="CM100" s="89" t="s">
-        <v>532</v>
+        <v>531</v>
       </c>
       <c r="CN100" s="82" t="s">
         <v>263</v>
@@ -39618,7 +39619,7 @@
         <v>0</v>
       </c>
       <c r="CM101" s="89" t="s">
-        <v>533</v>
+        <v>532</v>
       </c>
       <c r="CN101" s="82" t="s">
         <v>264</v>
@@ -39797,7 +39798,7 @@
         <v>0</v>
       </c>
       <c r="CM102" s="89" t="s">
-        <v>534</v>
+        <v>533</v>
       </c>
       <c r="CN102" s="82" t="s">
         <v>265</v>
@@ -40149,7 +40150,7 @@
         <v>0</v>
       </c>
       <c r="CM104" s="89" t="s">
-        <v>535</v>
+        <v>534</v>
       </c>
       <c r="CN104" s="84" t="s">
         <v>373</v>
@@ -40322,7 +40323,7 @@
         <v>0</v>
       </c>
       <c r="CM105" s="89" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="CN105" s="82" t="s">
         <v>267</v>
@@ -40495,7 +40496,7 @@
         <v>0</v>
       </c>
       <c r="CM106" s="89" t="s">
-        <v>536</v>
+        <v>535</v>
       </c>
       <c r="CN106" s="82" t="s">
         <v>268</v>
@@ -40674,7 +40675,7 @@
         <v>0</v>
       </c>
       <c r="CM107" s="89" t="s">
-        <v>537</v>
+        <v>536</v>
       </c>
       <c r="CN107" s="82" t="s">
         <v>269</v>
@@ -41024,7 +41025,7 @@
         <v>0</v>
       </c>
       <c r="CM109" s="89" t="s">
-        <v>538</v>
+        <v>537</v>
       </c>
       <c r="CN109" s="82" t="s">
         <v>271</v>
@@ -41197,7 +41198,7 @@
         <v>0</v>
       </c>
       <c r="CM110" s="89" t="s">
-        <v>564</v>
+        <v>563</v>
       </c>
       <c r="CN110" s="82" t="s">
         <v>272</v>
@@ -41372,7 +41373,7 @@
         <v>0</v>
       </c>
       <c r="CM111" s="89" t="s">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="CN111" s="82" t="s">
         <v>273</v>
@@ -41899,7 +41900,7 @@
         <v>0</v>
       </c>
       <c r="CM114" s="89" t="s">
-        <v>540</v>
+        <v>539</v>
       </c>
       <c r="CN114" s="82" t="s">
         <v>276</v>
@@ -42078,7 +42079,7 @@
         <v>0</v>
       </c>
       <c r="CM115" s="89" t="s">
-        <v>541</v>
+        <v>540</v>
       </c>
       <c r="CN115" s="82" t="s">
         <v>277</v>
@@ -42255,7 +42256,7 @@
         <v>0</v>
       </c>
       <c r="CM116" s="89" t="s">
-        <v>542</v>
+        <v>541</v>
       </c>
       <c r="CN116" s="82" t="s">
         <v>278</v>
@@ -42432,7 +42433,7 @@
         <v>0</v>
       </c>
       <c r="CM117" s="89" t="s">
-        <v>543</v>
+        <v>542</v>
       </c>
       <c r="CN117" s="82" t="s">
         <v>279</v>
@@ -42611,7 +42612,7 @@
         <v>0</v>
       </c>
       <c r="CM118" s="89" t="s">
-        <v>544</v>
+        <v>543</v>
       </c>
       <c r="CN118" s="82" t="s">
         <v>280</v>
@@ -42790,7 +42791,7 @@
         <v>0</v>
       </c>
       <c r="CM119" s="89" t="s">
-        <v>545</v>
+        <v>544</v>
       </c>
       <c r="CN119" s="82" t="s">
         <v>281</v>
@@ -44198,7 +44199,7 @@
         <v>0</v>
       </c>
       <c r="CM127" s="89" t="s">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="CN127" s="82" t="s">
         <v>289</v>
@@ -44375,7 +44376,7 @@
         <v>0</v>
       </c>
       <c r="CM128" s="89" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="CN128" s="82" t="s">
         <v>290</v>
@@ -44731,7 +44732,7 @@
         <v>0</v>
       </c>
       <c r="CM130" s="89" t="s">
-        <v>548</v>
+        <v>547</v>
       </c>
       <c r="CN130" s="82" t="s">
         <v>292</v>
@@ -44910,7 +44911,7 @@
         <v>0</v>
       </c>
       <c r="CM131" s="89" t="s">
-        <v>549</v>
+        <v>548</v>
       </c>
       <c r="CN131" s="82" t="s">
         <v>293</v>
@@ -45087,7 +45088,7 @@
         <v>0</v>
       </c>
       <c r="CM132" s="89" t="s">
-        <v>550</v>
+        <v>549</v>
       </c>
       <c r="CN132" s="82" t="s">
         <v>294</v>
@@ -46147,7 +46148,7 @@
         <v>0</v>
       </c>
       <c r="CM138" s="89" t="s">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="CN138" s="82" t="s">
         <v>300</v>
@@ -46845,7 +46846,7 @@
         <v>0</v>
       </c>
       <c r="CM142" s="89" t="s">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="CN142" s="82" t="s">
         <v>303</v>
@@ -47553,7 +47554,7 @@
         <v>0</v>
       </c>
       <c r="CM146" s="89" t="s">
-        <v>552</v>
+        <v>551</v>
       </c>
       <c r="CN146" s="82" t="s">
         <v>307</v>
@@ -47730,7 +47731,7 @@
         <v>0</v>
       </c>
       <c r="CM147" s="89" t="s">
-        <v>553</v>
+        <v>552</v>
       </c>
       <c r="CN147" s="82" t="s">
         <v>308</v>
@@ -47907,7 +47908,7 @@
         <v>0</v>
       </c>
       <c r="CM148" s="89" t="s">
-        <v>554</v>
+        <v>553</v>
       </c>
       <c r="CN148" s="82" t="s">
         <v>309</v>
@@ -48788,7 +48789,7 @@
         <v>0</v>
       </c>
       <c r="CM153" s="89" t="s">
-        <v>555</v>
+        <v>554</v>
       </c>
       <c r="CN153" s="82" t="s">
         <v>314</v>
@@ -51089,47 +51090,47 @@
       <c r="B2" s="30" t="s">
         <v>409</v>
       </c>
-      <c r="C2" s="30" t="s">
-        <v>447</v>
+      <c r="C2" s="30">
+        <v>1</v>
       </c>
       <c r="D2" s="32" t="s">
         <v>406</v>
       </c>
       <c r="E2" s="33" t="s">
-        <v>459</v>
+        <v>458</v>
       </c>
       <c r="F2" s="71"/>
     </row>
     <row r="3" spans="1:6">
       <c r="B3" s="29"/>
-      <c r="C3" s="30" t="s">
-        <v>447</v>
+      <c r="C3" s="30">
+        <v>1</v>
       </c>
       <c r="D3" s="32" t="s">
         <v>407</v>
       </c>
       <c r="E3" s="33" t="s">
-        <v>460</v>
+        <v>459</v>
       </c>
       <c r="F3" s="71"/>
     </row>
     <row r="4" spans="1:6">
       <c r="B4" s="29"/>
-      <c r="C4" s="30" t="s">
-        <v>447</v>
+      <c r="C4" s="30">
+        <v>1</v>
       </c>
       <c r="D4" s="32" t="s">
         <v>408</v>
       </c>
       <c r="E4" s="33" t="s">
-        <v>461</v>
+        <v>460</v>
       </c>
       <c r="F4" s="71"/>
     </row>
     <row r="5" spans="1:6">
       <c r="B5" s="29"/>
-      <c r="C5" s="30" t="s">
-        <v>447</v>
+      <c r="C5" s="30">
+        <v>1</v>
       </c>
       <c r="D5" s="32" t="s">
         <v>411</v>
@@ -51143,7 +51144,7 @@
     </row>
     <row r="6" spans="1:6">
       <c r="A6" s="128" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="B6" s="68" t="s">
         <v>378</v>
@@ -51158,7 +51159,7 @@
         <v>410</v>
       </c>
       <c r="F6" s="72" t="s">
-        <v>458</v>
+        <v>457</v>
       </c>
     </row>
     <row r="7" spans="1:6">
@@ -51171,7 +51172,7 @@
         <v>2</v>
       </c>
       <c r="E7" s="33" t="s">
-        <v>462</v>
+        <v>461</v>
       </c>
       <c r="F7" s="72"/>
     </row>
@@ -51185,7 +51186,7 @@
         <v>3</v>
       </c>
       <c r="E8" s="33" t="s">
-        <v>463</v>
+        <v>462</v>
       </c>
       <c r="F8" s="71"/>
     </row>
@@ -51261,13 +51262,13 @@
         <v>8</v>
       </c>
       <c r="E13" s="33" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="F13" s="71"/>
     </row>
     <row r="14" spans="1:6">
       <c r="A14" s="133" t="s">
-        <v>452</v>
+        <v>451</v>
       </c>
       <c r="B14" s="60" t="s">
         <v>380</v>
@@ -51377,7 +51378,7 @@
     </row>
     <row r="21" spans="1:6">
       <c r="A21" s="130" t="s">
-        <v>448</v>
+        <v>447</v>
       </c>
       <c r="B21" s="53" t="s">
         <v>382</v>
@@ -51389,7 +51390,7 @@
         <v>16</v>
       </c>
       <c r="E21" s="33" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="F21" s="71"/>
     </row>
@@ -51403,7 +51404,7 @@
         <v>17</v>
       </c>
       <c r="E22" s="33" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="F22" s="72"/>
     </row>
@@ -51417,7 +51418,7 @@
         <v>18</v>
       </c>
       <c r="E23" s="33" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="F23" s="72" t="s">
         <v>403</v>
@@ -51435,7 +51436,7 @@
         <v>19</v>
       </c>
       <c r="E24" s="33" t="s">
-        <v>454</v>
+        <v>453</v>
       </c>
       <c r="F24" s="72"/>
     </row>
@@ -51449,7 +51450,7 @@
         <v>20</v>
       </c>
       <c r="E25" s="33" t="s">
-        <v>455</v>
+        <v>454</v>
       </c>
       <c r="F25" s="72"/>
     </row>
@@ -51463,7 +51464,7 @@
         <v>21</v>
       </c>
       <c r="E26" s="33" t="s">
-        <v>456</v>
+        <v>455</v>
       </c>
       <c r="F26" s="72" t="s">
         <v>403</v>
@@ -51471,7 +51472,7 @@
     </row>
     <row r="27" spans="1:6">
       <c r="A27" s="132" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="B27" s="64" t="s">
         <v>384</v>
@@ -51545,13 +51546,13 @@
         <v>26</v>
       </c>
       <c r="E31" s="33" t="s">
-        <v>464</v>
+        <v>463</v>
       </c>
       <c r="F31" s="71"/>
     </row>
     <row r="32" spans="1:6">
       <c r="A32" s="134" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="B32" s="77" t="s">
         <v>386</v>
@@ -51563,7 +51564,7 @@
         <v>27</v>
       </c>
       <c r="E32" s="33" t="s">
-        <v>465</v>
+        <v>464</v>
       </c>
       <c r="F32" s="71"/>
     </row>
@@ -51577,7 +51578,7 @@
         <v>28</v>
       </c>
       <c r="E33" s="33" t="s">
-        <v>466</v>
+        <v>465</v>
       </c>
       <c r="F33" s="71"/>
     </row>
@@ -51591,7 +51592,7 @@
         <v>29</v>
       </c>
       <c r="E34" s="33" t="s">
-        <v>467</v>
+        <v>466</v>
       </c>
       <c r="F34" s="71"/>
     </row>
@@ -51607,7 +51608,7 @@
         <v>30</v>
       </c>
       <c r="E35" s="33" t="s">
-        <v>468</v>
+        <v>467</v>
       </c>
       <c r="F35" s="71"/>
     </row>
@@ -51671,7 +51672,7 @@
     </row>
     <row r="40" spans="1:6">
       <c r="A40" s="129" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B40" s="70" t="s">
         <v>389</v>
@@ -51700,7 +51701,7 @@
         <v>437</v>
       </c>
       <c r="F41" s="72" t="s">
-        <v>457</v>
+        <v>456</v>
       </c>
     </row>
     <row r="42" spans="1:6">
@@ -51727,7 +51728,7 @@
         <v>38</v>
       </c>
       <c r="E43" s="33" t="s">
-        <v>469</v>
+        <v>468</v>
       </c>
       <c r="F43" s="71"/>
     </row>
@@ -51747,7 +51748,7 @@
     </row>
     <row r="45" spans="1:6">
       <c r="A45" s="132" t="s">
-        <v>451</v>
+        <v>450</v>
       </c>
       <c r="B45" s="64" t="s">
         <v>390</v>
@@ -51807,7 +51808,7 @@
     </row>
     <row r="49" spans="1:6">
       <c r="A49" s="131" t="s">
-        <v>450</v>
+        <v>449</v>
       </c>
       <c r="B49" s="57" t="s">
         <v>391</v>
@@ -51819,7 +51820,7 @@
         <v>44</v>
       </c>
       <c r="E49" s="33" t="s">
-        <v>470</v>
+        <v>469</v>
       </c>
       <c r="F49" s="71"/>
     </row>
@@ -51833,7 +51834,7 @@
         <v>45</v>
       </c>
       <c r="E50" s="33" t="s">
-        <v>471</v>
+        <v>470</v>
       </c>
       <c r="F50" s="71"/>
     </row>
@@ -51847,7 +51848,7 @@
         <v>46</v>
       </c>
       <c r="E51" s="33" t="s">
-        <v>472</v>
+        <v>471</v>
       </c>
       <c r="F51" s="71"/>
     </row>
@@ -51861,7 +51862,7 @@
         <v>47</v>
       </c>
       <c r="E52" s="33" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="F52" s="71"/>
     </row>
@@ -51875,7 +51876,7 @@
         <v>48</v>
       </c>
       <c r="E53" s="33" t="s">
-        <v>474</v>
+        <v>473</v>
       </c>
       <c r="F53" s="71"/>
     </row>
@@ -51891,7 +51892,7 @@
         <v>49</v>
       </c>
       <c r="E54" s="33" t="s">
-        <v>475</v>
+        <v>474</v>
       </c>
       <c r="F54" s="71"/>
     </row>
@@ -51905,7 +51906,7 @@
         <v>50</v>
       </c>
       <c r="E55" s="33" t="s">
-        <v>476</v>
+        <v>475</v>
       </c>
       <c r="F55" s="71"/>
     </row>
@@ -51919,7 +51920,7 @@
         <v>51</v>
       </c>
       <c r="E56" s="33" t="s">
-        <v>477</v>
+        <v>476</v>
       </c>
       <c r="F56" s="71"/>
     </row>
@@ -51933,7 +51934,7 @@
         <v>52</v>
       </c>
       <c r="E57" s="33" t="s">
-        <v>478</v>
+        <v>477</v>
       </c>
       <c r="F57" s="71"/>
     </row>
@@ -51947,13 +51948,13 @@
         <v>53</v>
       </c>
       <c r="E58" s="33" t="s">
-        <v>473</v>
+        <v>472</v>
       </c>
       <c r="F58" s="71"/>
     </row>
     <row r="59" spans="1:6">
       <c r="A59" s="134" t="s">
-        <v>485</v>
+        <v>484</v>
       </c>
       <c r="B59" s="78" t="s">
         <v>404</v>
@@ -51965,7 +51966,7 @@
         <v>54</v>
       </c>
       <c r="E59" s="33" t="s">
-        <v>479</v>
+        <v>478</v>
       </c>
       <c r="F59" s="71"/>
     </row>
@@ -51979,7 +51980,7 @@
         <v>55</v>
       </c>
       <c r="E60" s="33" t="s">
-        <v>480</v>
+        <v>479</v>
       </c>
       <c r="F60" s="71"/>
     </row>
@@ -51995,7 +51996,7 @@
         <v>56</v>
       </c>
       <c r="E61" s="33" t="s">
-        <v>481</v>
+        <v>480</v>
       </c>
       <c r="F61" s="71"/>
     </row>
@@ -52009,13 +52010,13 @@
         <v>57</v>
       </c>
       <c r="E62" s="33" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="F62" s="71"/>
     </row>
     <row r="63" spans="1:6">
       <c r="A63" s="128" t="s">
-        <v>453</v>
+        <v>452</v>
       </c>
       <c r="B63" s="69" t="s">
         <v>394</v>
@@ -52027,7 +52028,7 @@
         <v>58</v>
       </c>
       <c r="E63" s="33" t="s">
-        <v>483</v>
+        <v>482</v>
       </c>
       <c r="F63" s="71"/>
     </row>
@@ -52041,13 +52042,13 @@
         <v>59</v>
       </c>
       <c r="E64" s="33" t="s">
-        <v>484</v>
+        <v>483</v>
       </c>
       <c r="F64" s="71"/>
     </row>
     <row r="65" spans="1:6">
       <c r="A65" s="129" t="s">
-        <v>449</v>
+        <v>448</v>
       </c>
       <c r="B65" s="55" t="s">
         <v>395</v>

</xml_diff>